<commit_message>
add: upload Excel template file (public/template.xlsx)
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twayair\training-record-webapp\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\백업\TEST\3. training-record-streamlit\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B29FB0C-EAE4-4CAA-88F1-3EAD472A60AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322FEB50-3959-412C-80D9-40A5CFCF6FF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -161,7 +161,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -230,118 +230,195 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -365,15 +442,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>119530</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>52295</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>287019</xdr:colOff>
+      <xdr:colOff>406549</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>416559</xdr:rowOff>
+      <xdr:rowOff>468854</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -402,8 +479,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="985519" cy="416559"/>
+          <a:off x="119530" y="52295"/>
+          <a:ext cx="1093843" cy="416559"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -715,380 +792,380 @@
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="1.09765625" customWidth="1"/>
     <col min="8" max="8" width="15.09765625" customWidth="1"/>
-    <col min="9" max="9" width="8" customWidth="1"/>
+    <col min="9" max="9" width="8.69921875" customWidth="1"/>
     <col min="10" max="10" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
     </row>
     <row r="3" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="5"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="19"/>
     </row>
     <row r="4" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="8"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="22"/>
     </row>
     <row r="5" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="11" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="12"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="11" t="s">
+      <c r="E5" s="24"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="12"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="10"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="14"/>
     </row>
     <row r="6" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="16"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="12"/>
     </row>
     <row r="7" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="17" t="s">
+      <c r="B7" s="13"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="18"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="17" t="s">
+      <c r="E7" s="16"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="18"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="10"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="14"/>
     </row>
     <row r="8" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="21" t="s">
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-      <c r="J8" s="22"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="29"/>
     </row>
     <row r="9" spans="1:10" ht="23" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="17" t="s">
+      <c r="B9" s="31"/>
+      <c r="C9" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="17" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="17" t="s">
+      <c r="F9" s="32"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="I9" s="18"/>
-      <c r="J9" s="2" t="s">
+      <c r="I9" s="31"/>
+      <c r="J9" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="13"/>
-    </row>
-    <row r="11" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="13"/>
-    </row>
-    <row r="12" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="13"/>
-    </row>
-    <row r="13" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="13"/>
-    </row>
-    <row r="14" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="13"/>
-    </row>
-    <row r="15" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="13"/>
-    </row>
-    <row r="16" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="13"/>
-    </row>
-    <row r="17" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="13"/>
-    </row>
-    <row r="18" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="13"/>
-    </row>
-    <row r="19" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="13"/>
-    </row>
-    <row r="20" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="9"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="13"/>
-    </row>
-    <row r="21" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="13"/>
-    </row>
-    <row r="22" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="9"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="13"/>
-    </row>
-    <row r="23" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="9"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="13"/>
-    </row>
-    <row r="24" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="13"/>
-    </row>
-    <row r="25" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="25" t="s">
+    <row r="10" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="13"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="13"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="13"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="13"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="13"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="13"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="13"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="13"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="13"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="13"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="13"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="13"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="13"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="13"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="25"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="27"/>
+      <c r="B25" s="39"/>
+      <c r="C25" s="39"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="39"/>
+      <c r="I25" s="39"/>
+      <c r="J25" s="40"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="25" t="s">
+      <c r="A26" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="26"/>
-      <c r="J26" s="27"/>
-    </row>
-    <row r="27" spans="1:10" ht="82" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="28" t="s">
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="35"/>
+    </row>
+    <row r="27" spans="1:10" ht="40" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="30" t="s">
+      <c r="B27" s="37"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="I27" s="24"/>
-      <c r="J27" s="10"/>
+      <c r="I27" s="41"/>
+      <c r="J27" s="42"/>
     </row>
     <row r="28" spans="1:10" ht="17" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="32" t="s">
+      <c r="A28" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="34" t="s">
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="35" t="s">
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1181,7 +1258,7 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="92" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="91" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>